<commit_message>
feat: overlay Tạm dừng bám design (toggle nhanh + Cài đặt phủ) cho Endless & Campaign
Overlay Tạm dừng làm đúng pause-screen.jsx: hàng toggle nhanh Âm thanh·Nhạc
(component GjQuickToggle mới), CTA TIẾP TỤC, hàng Chơi lại·Cài đặt, nút thoát
(Về Home / Danh sách màn); dismissable=false. "Cài đặt" mở SettingsScreen phủ
toàn màn thay vì đổi route → giữ nguyên ván đang chơi. Nối settings/onSound/
onMusic/onVibrate từ MainActivity xuống EndlessPlayScreen & CampaignPlayScreen.

Gộp thêm tiến độ MVP đang dang dở trong cây làm việc: prototype Campaign
(chọn màn · intro · chơi · màn thắng), hệ dạy luật + Cẩm nang, cập nhật
design system + docs + assets. Bỏ theo dõi core/bin (thêm vào .gitignore).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/level-design-100-levels.xlsx
+++ b/docs/level-design-100-levels.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -212,6 +212,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -578,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S101"/>
+  <dimension ref="A1:T101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -600,6 +606,7 @@
     <col width="7" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="30" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -698,6 +705,11 @@
           <t>Cơ chế mới (đầu world)</t>
         </is>
       </c>
+      <c r="T1" s="26" t="inlineStr">
+        <is>
+          <t>goal_type (code)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -715,7 +727,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Cỏ 1</t>
+          <t>Hàng đầu tiên</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -725,16 +737,16 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Xóa hàng</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Xóa 1 hàng ngang đầu tiên (bàn trống, tự xây)</t>
         </is>
       </c>
       <c r="H2" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I2" s="5" t="n">
         <v>0</v>
@@ -746,10 +758,10 @@
         <v>0</v>
       </c>
       <c r="L2" s="5" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M2" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
@@ -757,20 +769,25 @@
         </is>
       </c>
       <c r="O2" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P2" s="5" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="Q2" s="5" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="R2" s="5" t="n">
         <v>1</v>
       </c>
       <c r="S2" s="4" t="inlineStr">
         <is>
-          <t>Đặt mảnh + xóa hàng/cột (dạy cơ bản)</t>
+          <t>Đặt mảnh + xóa HÀNG (dạy cơ bản)</t>
+        </is>
+      </c>
+      <c r="T2" s="27" t="inlineStr">
+        <is>
+          <t>CLEAR_ROW_FIRST</t>
         </is>
       </c>
     </row>
@@ -790,7 +807,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Cỏ 2</t>
+          <t>Cột đầu tiên</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -800,16 +817,16 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Xóa cột</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Xóa 1 cột dọc (chồng 3 V3 cùng cột)</t>
         </is>
       </c>
       <c r="H3" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I3" s="5" t="n">
         <v>0</v>
@@ -821,29 +838,38 @@
         <v>0</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M3" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>Nước</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P3" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q3" s="5" t="n">
         <v>5</v>
-      </c>
-      <c r="N3" s="5" t="inlineStr">
-        <is>
-          <t>Nước</t>
-        </is>
-      </c>
-      <c r="O3" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="P3" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q3" s="5" t="n">
-        <v>9</v>
       </c>
       <c r="R3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="S3" s="4" t="inlineStr"/>
+      <c r="S3" s="4" t="inlineStr">
+        <is>
+          <t>Xóa CỘT (khay mảnh dọc)</t>
+        </is>
+      </c>
+      <c r="T3" s="27" t="inlineStr">
+        <is>
+          <t>CLEAR_COL_FIRST</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -861,7 +887,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Cỏ 3</t>
+          <t>Cú xoay đầu</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -871,19 +897,19 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Xoay trọng lực</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Thực hiện 1 cú xoay — preset nhỏ: xoay lùa ô lạc lấp lỗ cột → xóa cột (⚠ chơi thử)</t>
         </is>
       </c>
       <c r="H4" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -895,26 +921,35 @@
         <v>11</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Xoay</t>
         </is>
       </c>
       <c r="O4" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P4" s="5" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="Q4" s="5" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="R4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="S4" s="4" t="inlineStr"/>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>Xoay trọng lực — cơ chế chữ ký</t>
+        </is>
+      </c>
+      <c r="T4" s="27" t="inlineStr">
+        <is>
+          <t>ROTATE_FIRST</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -932,29 +967,29 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Cỏ 4</t>
+          <t>Siêu khối</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Thường</t>
+          <t>Tutorial</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Ghép siêu khối 1</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Gộp 9 ô cùng màu → siêu khối cấp 1</t>
         </is>
       </c>
       <c r="H5" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" s="5" t="n">
         <v>0</v>
@@ -963,29 +998,38 @@
         <v>0</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="M5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>Nước</t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q5" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="N5" s="5" t="inlineStr">
-        <is>
-          <t>Nước</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="P5" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q5" s="5" t="n">
-        <v>9</v>
-      </c>
       <c r="R5" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="S5" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>Siêu khối cấp 1 (merge-9)</t>
+        </is>
+      </c>
+      <c r="T5" s="27" t="inlineStr">
+        <is>
+          <t>MAKE_SUPER1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1003,29 +1047,29 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Cỏ 5</t>
+          <t>Đại nổ</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Thường</t>
+          <t>Tutorial</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Ghép siêu khối 2</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Gộp thành siêu khối cấp 2 (đại nổ)</t>
         </is>
       </c>
       <c r="H6" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -1034,7 +1078,7 @@
         <v>0</v>
       </c>
       <c r="L6" s="5" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="M6" s="5" t="n">
         <v>5</v>
@@ -1054,9 +1098,18 @@
         <v>9</v>
       </c>
       <c r="R6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="S6" s="4" t="inlineStr"/>
+        <v>2.5</v>
+      </c>
+      <c r="S6" s="4" t="inlineStr">
+        <is>
+          <t>Siêu khối cấp 2 (B4 đại nổ)</t>
+        </is>
+      </c>
+      <c r="T6" s="27" t="inlineStr">
+        <is>
+          <t>MAKE_SUPER2</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1074,29 +1127,29 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Cỏ 6</t>
+          <t>Cầu vồng 1</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Breather</t>
+          <t>Tutorial</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Tạo cầu vồng</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Tạo ô cầu vồng đầu tiên (3×3 ba màu sọc)</t>
         </is>
       </c>
       <c r="H7" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>0</v>
@@ -1105,29 +1158,38 @@
         <v>0</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="M7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>Nước</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="N7" s="5" t="inlineStr">
-        <is>
-          <t>Nước</t>
-        </is>
-      </c>
-      <c r="O7" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="P7" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q7" s="5" t="n">
-        <v>9</v>
-      </c>
       <c r="R7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="S7" s="4" t="inlineStr"/>
+        <v>2.5</v>
+      </c>
+      <c r="S7" s="4" t="inlineStr">
+        <is>
+          <t>Ô cầu vồng (wild) — 3×3 ba màu</t>
+        </is>
+      </c>
+      <c r="T7" s="27" t="inlineStr">
+        <is>
+          <t>MAKE_RAINBOW</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1145,7 +1207,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Cỏ 7</t>
+          <t>Cầu vồng 2</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1155,19 +1217,19 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Cầu vồng super</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Tạo 1 cầu vồng siêu cấp (LIỆU NGHIỆM CAO)</t>
         </is>
       </c>
       <c r="H8" s="5" t="n">
         <v>6</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -1176,7 +1238,7 @@
         <v>0</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="M8" s="5" t="n">
         <v>6</v>
@@ -1196,9 +1258,18 @@
         <v>10</v>
       </c>
       <c r="R8" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="S8" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>Cầu vồng super — cần chơi thử</t>
+        </is>
+      </c>
+      <c r="T8" s="27" t="inlineStr">
+        <is>
+          <t>MAKE_RAINBOW_SUPER</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1216,29 +1287,29 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Cỏ 8</t>
+          <t>Combo x2 đầu tiên</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Thường</t>
+          <t>Tutorial</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Combo ×2</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Đạt combo ×2 lần đầu (xóa ≥2 hàng/cột 1 nước)</t>
         </is>
       </c>
       <c r="H9" s="5" t="n">
         <v>6</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J9" s="5" t="n">
         <v>0</v>
@@ -1247,29 +1318,38 @@
         <v>0</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="M9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>Nước</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="P9" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="N9" s="5" t="inlineStr">
-        <is>
-          <t>Nước</t>
-        </is>
-      </c>
-      <c r="O9" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="P9" s="5" t="n">
-        <v>8</v>
-      </c>
       <c r="Q9" s="5" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="R9" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="S9" s="4" t="inlineStr"/>
+        <v>2.5</v>
+      </c>
+      <c r="S9" s="4" t="inlineStr">
+        <is>
+          <t>Combo ×2 — dạy dồn chuỗi</t>
+        </is>
+      </c>
+      <c r="T9" s="27" t="inlineStr">
+        <is>
+          <t>COMBO_X2</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1287,29 +1367,29 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Cỏ 9</t>
+          <t>Hai trăm điểm</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Thường</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Đạt điểm</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Đạt 200 điểm để qua màn</t>
         </is>
       </c>
       <c r="H10" s="5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -1318,29 +1398,40 @@
         <v>0</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="M10" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O10" s="5" t="n">
-        <v>6</v>
+        <v>360</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>8</v>
+        <v>280</v>
       </c>
       <c r="Q10" s="5" t="n">
-        <v>10</v>
+        <v>200</v>
       </c>
       <c r="R10" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="S10" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="S10" s="4" t="inlineStr">
+        <is>
+          <t>Chơi lấy điểm (ngưỡng 200)</t>
+        </is>
+      </c>
+      <c r="T10" s="27" t="inlineStr">
+        <is>
+          <t>REACH_SCORE</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1358,7 +1449,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Cỏ 10</t>
+          <t>Boss Combo</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1368,19 +1459,19 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Boss combo</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Bào 5 máu boss; mỗi combo ≥×2 gây (bậc−1) sát thương</t>
         </is>
       </c>
       <c r="H11" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J11" s="5" t="n">
         <v>2</v>
@@ -1389,29 +1480,40 @@
         <v>0</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="M11" s="5" t="n">
-        <v>7</v>
+        <v>0</v>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Combo</t>
         </is>
       </c>
       <c r="O11" s="5" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="Q11" s="5" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="R11" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="S11" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="S11" s="4" t="inlineStr">
+        <is>
+          <t>Boss bào máu bằng combo (máu=5)</t>
+        </is>
+      </c>
+      <c r="T11" s="27" t="inlineStr">
+        <is>
+          <t>BOSS_COMBO</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
@@ -1439,16 +1541,16 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Đạt điểm</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Đạt 250 điểm; cụm to rối — xoay để gỡ</t>
         </is>
       </c>
       <c r="H12" s="5" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I12" s="5" t="n">
         <v>1</v>
@@ -1460,31 +1562,38 @@
         <v>0</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="M12" s="5" t="n">
-        <v>7</v>
+        <v>14</v>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O12" s="5" t="n">
-        <v>7</v>
+        <v>450</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>9</v>
+        <v>320</v>
       </c>
       <c r="Q12" s="5" t="n">
-        <v>11</v>
+        <v>250</v>
       </c>
       <c r="R12" s="5" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="S12" s="4" t="inlineStr">
         <is>
-          <t>Vật lý cụm kẹt + cú xoay trọng lực đầu tiên</t>
+          <t>Cụm to rối — xoay gỡ kẹt (luyện lõi)</t>
+        </is>
+      </c>
+      <c r="T12" s="27" t="inlineStr">
+        <is>
+          <t>REACH_SCORE</t>
         </is>
       </c>
     </row>
@@ -1514,16 +1623,16 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Đạt điểm</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Đạt 300 điểm bằng cascade sau xoay</t>
         </is>
       </c>
       <c r="H13" s="5" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I13" s="5" t="n">
         <v>1</v>
@@ -1535,29 +1644,40 @@
         <v>0</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="M13" s="5" t="n">
-        <v>7</v>
+        <v>16</v>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O13" s="5" t="n">
-        <v>7</v>
+        <v>520</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>9</v>
+        <v>400</v>
       </c>
       <c r="Q13" s="5" t="n">
-        <v>11</v>
+        <v>300</v>
       </c>
       <c r="R13" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="S13" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="S13" s="4" t="inlineStr">
+        <is>
+          <t>Cascade dây chuyền sau xoay</t>
+        </is>
+      </c>
+      <c r="T13" s="27" t="inlineStr">
+        <is>
+          <t>REACH_SCORE</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
@@ -1585,16 +1705,16 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Phá gốc dây</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Phá 1 gốc dây leo (mọc chậm: 2 lượt/đốt)</t>
         </is>
       </c>
       <c r="H14" s="5" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I14" s="5" t="n">
         <v>1</v>
@@ -1603,13 +1723,13 @@
         <v>0</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M14" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
@@ -1617,18 +1737,27 @@
         </is>
       </c>
       <c r="O14" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q14" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="R14" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="S14" s="4" t="inlineStr"/>
+        <v>2.5</v>
+      </c>
+      <c r="S14" s="4" t="inlineStr">
+        <is>
+          <t>DÂY LEO mọc lan — giới thiệu; cắt gốc để diệt</t>
+        </is>
+      </c>
+      <c r="T14" s="27" t="inlineStr">
+        <is>
+          <t>CLEAR_TARGETS</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n">
@@ -1656,16 +1785,16 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Phá gốc dây</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Phá 2 gốc dây leo</t>
         </is>
       </c>
       <c r="H15" s="5" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>1</v>
@@ -1674,13 +1803,13 @@
         <v>0</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="M15" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
@@ -1688,18 +1817,27 @@
         </is>
       </c>
       <c r="O15" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q15" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R15" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="S15" s="4" t="inlineStr"/>
+        <v>2.5</v>
+      </c>
+      <c r="S15" s="4" t="inlineStr">
+        <is>
+          <t>Cắt gốc vs tỉa đốt</t>
+        </is>
+      </c>
+      <c r="T15" s="27" t="inlineStr">
+        <is>
+          <t>CLEAR_TARGETS</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
@@ -1727,50 +1865,61 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Hỗn hợp</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Phá 1 gốc + đạt 300 điểm</t>
         </is>
       </c>
       <c r="H16" s="5" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="M16" s="5" t="n">
-        <v>8</v>
+        <v>17</v>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O16" s="5" t="n">
-        <v>8</v>
+        <v>480</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>10</v>
+        <v>380</v>
       </c>
       <c r="Q16" s="5" t="n">
-        <v>12</v>
+        <v>300</v>
       </c>
       <c r="R16" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="S16" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="S16" s="4" t="inlineStr">
+        <is>
+          <t>Dây leo + điểm cùng lúc</t>
+        </is>
+      </c>
+      <c r="T16" s="27" t="inlineStr">
+        <is>
+          <t>MIXED</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
@@ -1798,16 +1947,16 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Ghép siêu khối 1</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Ghép 1 siêu khối (không dây leo) — màn thở</t>
         </is>
       </c>
       <c r="H17" s="5" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>2</v>
@@ -1822,7 +1971,7 @@
         <v>12</v>
       </c>
       <c r="M17" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="N17" s="5" t="inlineStr">
         <is>
@@ -1830,18 +1979,27 @@
         </is>
       </c>
       <c r="O17" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="Q17" s="5" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="R17" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="S17" s="4" t="inlineStr"/>
+        <v>1.5</v>
+      </c>
+      <c r="S17" s="4" t="inlineStr">
+        <is>
+          <t>Màn thở</t>
+        </is>
+      </c>
+      <c r="T17" s="27" t="inlineStr">
+        <is>
+          <t>MAKE_SUPER1</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
@@ -1869,31 +2027,31 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Phá gốc dây</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Phá 2 gốc (mọc nhanh: 1 lượt/đốt)</t>
         </is>
       </c>
       <c r="H18" s="5" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="M18" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
@@ -1901,18 +2059,27 @@
         </is>
       </c>
       <c r="O18" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q18" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R18" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="S18" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="S18" s="4" t="inlineStr">
+        <is>
+          <t>Dây leo mọc nhanh — áp lực nhịp độ</t>
+        </is>
+      </c>
+      <c r="T18" s="27" t="inlineStr">
+        <is>
+          <t>CLEAR_TARGETS</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n">
@@ -1940,50 +2107,61 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Đạt điểm</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Đạt 400 điểm giữa dây leo</t>
         </is>
       </c>
       <c r="H19" s="5" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="M19" s="5" t="n">
-        <v>8</v>
+        <v>19</v>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N19" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O19" s="5" t="n">
-        <v>8</v>
+        <v>620</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>10</v>
+        <v>500</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>12</v>
+        <v>400</v>
       </c>
       <c r="R19" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="S19" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="S19" s="4" t="inlineStr">
+        <is>
+          <t>Kiếm điểm giữa dây leo</t>
+        </is>
+      </c>
+      <c r="T19" s="27" t="inlineStr">
+        <is>
+          <t>REACH_SCORE</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
@@ -2011,50 +2189,61 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Hỗn hợp</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Phá 2 gốc + đạt 350 điểm</t>
         </is>
       </c>
       <c r="H20" s="5" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="M20" s="5" t="n">
-        <v>8</v>
+        <v>20</v>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O20" s="5" t="n">
-        <v>8</v>
+        <v>560</v>
       </c>
       <c r="P20" s="5" t="n">
-        <v>10</v>
+        <v>450</v>
       </c>
       <c r="Q20" s="5" t="n">
-        <v>12</v>
+        <v>350</v>
       </c>
       <c r="R20" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="S20" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="S20" s="4" t="inlineStr">
+        <is>
+          <t>Tổng hợp dây leo + điểm</t>
+        </is>
+      </c>
+      <c r="T20" s="27" t="inlineStr">
+        <is>
+          <t>MIXED</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n">
@@ -2082,22 +2271,22 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
+          <t>Boss combo</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Xóa hết khối trên bàn</t>
+          <t>Kẻ Đổ Rác (máu 8): đổ lá mỗi lượt; combo ≥×2 gây (bậc−1) sát thương</t>
         </is>
       </c>
       <c r="H21" s="5" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="I21" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J21" s="5" t="n">
         <v>0</v>
-      </c>
-      <c r="J21" s="5" t="n">
-        <v>2</v>
       </c>
       <c r="K21" s="5" t="n">
         <v>0</v>
@@ -2105,27 +2294,38 @@
       <c r="L21" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="M21" s="5" t="n">
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>Combo</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="P21" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q21" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="N21" s="5" t="inlineStr">
-        <is>
-          <t>Nước</t>
-        </is>
-      </c>
-      <c r="O21" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="P21" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q21" s="5" t="n">
-        <v>12</v>
-      </c>
       <c r="R21" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="S21" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="S21" s="4" t="inlineStr">
+        <is>
+          <t>Boss Kẻ Đổ Rác (DPS race)</t>
+        </is>
+      </c>
+      <c r="T21" s="27" t="inlineStr">
+        <is>
+          <t>BOSS_COMBO</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n">
@@ -2153,19 +2353,19 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Phá giọt nước</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 2 ô đích</t>
+          <t>Phá 2 giọt nước (dòng chảy nhẹ 1 dải)</t>
         </is>
       </c>
       <c r="H22" s="5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0</v>
@@ -2177,7 +2377,7 @@
         <v>16</v>
       </c>
       <c r="M22" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
@@ -2185,20 +2385,25 @@
         </is>
       </c>
       <c r="O22" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P22" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q22" s="5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="R22" s="5" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="S22" s="4" t="inlineStr">
         <is>
-          <t>Combo dây chuyền sau xoay + ô đích (giọt nước)</t>
+          <t>DÒNG CHẢY — ô trượt theo dòng (giới thiệu)</t>
+        </is>
+      </c>
+      <c r="T22" s="27" t="inlineStr">
+        <is>
+          <t>CLEAR_TARGETS</t>
         </is>
       </c>
     </row>
@@ -2228,50 +2433,61 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Đạt điểm</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 2 ô đích</t>
+          <t>Đạt 450 điểm bằng cascade dòng chảy</t>
         </is>
       </c>
       <c r="H23" s="5" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J23" s="5" t="n">
         <v>0</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L23" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="M23" s="5" t="n">
-        <v>8</v>
+        <v>16</v>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N23" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O23" s="5" t="n">
-        <v>8</v>
+        <v>700</v>
       </c>
       <c r="P23" s="5" t="n">
-        <v>10</v>
+        <v>560</v>
       </c>
       <c r="Q23" s="5" t="n">
-        <v>12</v>
+        <v>450</v>
       </c>
       <c r="R23" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="S23" s="4" t="inlineStr"/>
+        <v>2.5</v>
+      </c>
+      <c r="S23" s="4" t="inlineStr">
+        <is>
+          <t>Cascade dài nhờ dòng chảy</t>
+        </is>
+      </c>
+      <c r="T23" s="27" t="inlineStr">
+        <is>
+          <t>REACH_SCORE</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n">
@@ -2299,19 +2515,19 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Phá giọt nước</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 3 ô đích</t>
+          <t>Phá 3 giọt nước</t>
         </is>
       </c>
       <c r="H24" s="5" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0</v>
@@ -2340,9 +2556,18 @@
         <v>12</v>
       </c>
       <c r="R24" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="S24" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="S24" s="4" t="inlineStr">
+        <is>
+          <t>Nhiều giọt hơn</t>
+        </is>
+      </c>
+      <c r="T24" s="27" t="inlineStr">
+        <is>
+          <t>CLEAR_TARGETS</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="n">
@@ -2370,50 +2595,61 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Hỗn hợp</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 3 ô đích</t>
+          <t>Phá 2 giọt + đạt 400 điểm</t>
         </is>
       </c>
       <c r="H25" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J25" s="5" t="n">
         <v>0</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L25" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="M25" s="5" t="n">
-        <v>9</v>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N25" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O25" s="5" t="n">
-        <v>9</v>
+        <v>640</v>
       </c>
       <c r="P25" s="5" t="n">
-        <v>11</v>
+        <v>520</v>
       </c>
       <c r="Q25" s="5" t="n">
-        <v>13</v>
+        <v>400</v>
       </c>
       <c r="R25" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="S25" s="4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="S25" s="4" t="inlineStr">
+        <is>
+          <t>Giọt + điểm</t>
+        </is>
+      </c>
+      <c r="T25" s="27" t="inlineStr">
+        <is>
+          <t>MIXED</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n">
@@ -2441,31 +2677,31 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Phá giọt nước</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 3 ô đích</t>
+          <t>Phá 3 giọt CHÔN SÂU (đào bằng cascade)</t>
         </is>
       </c>
       <c r="H26" s="5" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K26" s="5" t="n">
         <v>3</v>
       </c>
       <c r="L26" s="5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M26" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
@@ -2473,18 +2709,27 @@
         </is>
       </c>
       <c r="O26" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P26" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q26" s="5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R26" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="S26" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="S26" s="4" t="inlineStr">
+        <is>
+          <t>Ô đích chôn sâu (E2) — dùng cascade lộ</t>
+        </is>
+      </c>
+      <c r="T26" s="27" t="inlineStr">
+        <is>
+          <t>CLEAR_TARGETS</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="n">
@@ -2512,16 +2757,16 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Đạt điểm</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 4 ô đích</t>
+          <t>Đạt 300 điểm (màn thở)</t>
         </is>
       </c>
       <c r="H27" s="5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I27" s="5" t="n">
         <v>2</v>
@@ -2530,32 +2775,43 @@
         <v>0</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L27" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="M27" s="5" t="n">
-        <v>9</v>
+        <v>13</v>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N27" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O27" s="5" t="n">
-        <v>9</v>
+        <v>480</v>
       </c>
       <c r="P27" s="5" t="n">
-        <v>11</v>
+        <v>380</v>
       </c>
       <c r="Q27" s="5" t="n">
-        <v>13</v>
+        <v>300</v>
       </c>
       <c r="R27" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="S27" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="S27" s="4" t="inlineStr">
+        <is>
+          <t>Màn thở</t>
+        </is>
+      </c>
+      <c r="T27" s="27" t="inlineStr">
+        <is>
+          <t>REACH_SCORE</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n">
@@ -2583,19 +2839,19 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Phá giọt nước</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 4 ô đích</t>
+          <t>Phá 4 giọt (dòng chảy mạnh 2 dải)</t>
         </is>
       </c>
       <c r="H28" s="5" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>1</v>
@@ -2604,10 +2860,10 @@
         <v>4</v>
       </c>
       <c r="L28" s="5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M28" s="5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
@@ -2615,18 +2871,27 @@
         </is>
       </c>
       <c r="O28" s="5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P28" s="5" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="Q28" s="5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="R28" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="S28" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="S28" s="4" t="inlineStr">
+        <is>
+          <t>Dòng chảy mạnh (2 dải)</t>
+        </is>
+      </c>
+      <c r="T28" s="27" t="inlineStr">
+        <is>
+          <t>CLEAR_TARGETS</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="n">
@@ -2654,50 +2919,61 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Đạt điểm</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 4 ô đích</t>
+          <t>Đạt 550 điểm</t>
         </is>
       </c>
       <c r="H29" s="5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J29" s="5" t="n">
         <v>1</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L29" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="M29" s="5" t="n">
-        <v>9</v>
+        <v>20</v>
+      </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N29" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O29" s="5" t="n">
-        <v>9</v>
+        <v>850</v>
       </c>
       <c r="P29" s="5" t="n">
-        <v>11</v>
+        <v>700</v>
       </c>
       <c r="Q29" s="5" t="n">
-        <v>13</v>
+        <v>550</v>
       </c>
       <c r="R29" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="S29" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="S29" s="4" t="inlineStr">
+        <is>
+          <t>Điểm cao giữa dòng</t>
+        </is>
+      </c>
+      <c r="T29" s="27" t="inlineStr">
+        <is>
+          <t>REACH_SCORE</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n">
@@ -2725,50 +3001,61 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Hỗn hợp</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 5 ô đích</t>
+          <t>Phá 3 giọt + đạt 450 điểm</t>
         </is>
       </c>
       <c r="H30" s="5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J30" s="5" t="n">
         <v>1</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="M30" s="5" t="n">
-        <v>9</v>
+        <v>20</v>
+      </c>
+      <c r="M30" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O30" s="5" t="n">
-        <v>9</v>
+        <v>720</v>
       </c>
       <c r="P30" s="5" t="n">
-        <v>11</v>
+        <v>580</v>
       </c>
       <c r="Q30" s="5" t="n">
-        <v>13</v>
+        <v>450</v>
       </c>
       <c r="R30" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="S30" s="4" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="S30" s="4" t="inlineStr">
+        <is>
+          <t>Tổng hợp giọt + điểm</t>
+        </is>
+      </c>
+      <c r="T30" s="27" t="inlineStr">
+        <is>
+          <t>MIXED</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="n">
@@ -2796,50 +3083,61 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Boss combo</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 6 ô đích</t>
+          <t>Thần Thác (máu 10): đảo trọng lực/dòng mỗi 3 lượt; combo ≥×2 gây (bậc−1) sát thương</t>
         </is>
       </c>
       <c r="H31" s="5" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J31" s="5" t="n">
         <v>3</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L31" s="5" t="n">
-        <v>23</v>
-      </c>
-      <c r="M31" s="5" t="n">
-        <v>9</v>
+        <v>20</v>
+      </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N31" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Combo</t>
         </is>
       </c>
       <c r="O31" s="5" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="P31" s="5" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="Q31" s="5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="R31" s="5" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="S31" s="4" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="S31" s="4" t="inlineStr">
+        <is>
+          <t>Boss Thần Thác (Tham Trọng Lực)</t>
+        </is>
+      </c>
+      <c r="T31" s="27" t="inlineStr">
+        <is>
+          <t>BOSS_COMBO</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="12" t="n">
@@ -7928,16 +8226,18 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Đặt mảnh + xóa hàng/cột (dạy cơ bản)</t>
+          <t>TUTORIAL WORLD — dạy tất cả: xóa hàng/cột → xoay → siêu khối 1&amp;2 → cầu vồng 1&amp;2 → combo ×2 → boss</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="n">
-        <v>0</v>
+          <t>Tutorial + Điểm + Boss</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>0–3</t>
+        </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
@@ -7968,16 +8268,18 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Vật lý cụm kẹt + cú xoay trọng lực đầu tiên</t>
+          <t>DÂY LEO mọc lan (bám cứng, cắt gốc để diệt) + luyện cụm kẹt/xoay</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Dọn sạch</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="n">
-        <v>1</v>
+          <t>Điểm + Phá gốc dây + Boss</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>1–3</t>
+        </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
@@ -8008,16 +8310,18 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Combo dây chuyền sau xoay + ô đích (giọt nước)</t>
+          <t>DÒNG CHẢY (ô trượt theo dòng) + ô đích giọt nước (có chôn sâu) — nhấn cascade dài</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>1</v>
+          <t>Giọt nước + Điểm + Boss</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>2–4</t>
+        </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: redesign W2 (vine MINT-only + boss Thần Rừng) & W3 (thác nước BFS + boss Thần Thác)
- :core — quy tắc MINT-only phá gốc vine (Resolve.kt + SuperBlock.kt);
  WaterfallFlow module (BFS chảy/tách/ngập/phá giọt); boss vine spawn;
  CampaignLevels L11-L30 viết lại; CampaignSolver hỗ trợ flooded cells
- :app — RE-SKIN Home/Cẩm nang/Campaign/Result; ObjectiveBar; LevelFailScreen;
  W2/W3 map + assets; design system cập nhật
- :game — mắt tính cách màu; JellyDraw hiệu ứng; LivingJelly nâng cấp
- Tests: VineTest MINT rule, WaterfallFlowTest, CampaignLevelsTest cấu trúc W2/W3

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/level-design-100-levels.xlsx
+++ b/docs/level-design-100-levels.xlsx
@@ -3165,16 +3165,16 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Đạt điểm</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 3 ô đích</t>
+          <t>Đạt 500 điểm (đá cố định chia bàn)</t>
         </is>
       </c>
       <c r="H32" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I32" s="5" t="n">
         <v>2</v>
@@ -3183,34 +3183,41 @@
         <v>2</v>
       </c>
       <c r="K32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="M32" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t>Điểm</t>
+        </is>
+      </c>
+      <c r="O32" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="P32" s="5" t="n">
+        <v>620</v>
+      </c>
+      <c r="Q32" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="R32" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="L32" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="M32" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="N32" s="5" t="inlineStr">
-        <is>
-          <t>Nước</t>
-        </is>
-      </c>
-      <c r="O32" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="P32" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q32" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="R32" s="5" t="n">
-        <v>2</v>
-      </c>
       <c r="S32" s="4" t="inlineStr">
         <is>
-          <t>Đá cố định làm chướng ngại</t>
+          <t>ĐÁ CỐ ĐỊNH — chướng ngại chia bàn (giới thiệu)</t>
+        </is>
+      </c>
+      <c r="T32" s="27" t="inlineStr">
+        <is>
+          <t>REACH_SCORE</t>
         </is>
       </c>
     </row>
@@ -3240,50 +3247,59 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Phá cổ vật</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 3 ô đích</t>
+          <t>Phá 2 cổ vật (bị đá vây)</t>
         </is>
       </c>
       <c r="H33" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I33" s="5" t="n">
         <v>2</v>
       </c>
       <c r="J33" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="K33" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="K33" s="5" t="n">
+      <c r="L33" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="M33" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>Nước</t>
+        </is>
+      </c>
+      <c r="O33" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="P33" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q33" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="R33" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="L33" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="M33" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="N33" s="5" t="inlineStr">
-        <is>
-          <t>Nước</t>
-        </is>
-      </c>
-      <c r="O33" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="P33" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q33" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="R33" s="5" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="S33" s="4" t="inlineStr"/>
+      <c r="S33" s="4" t="inlineStr">
+        <is>
+          <t>Cổ vật bị đá vây — xoay để tiếp cận</t>
+        </is>
+      </c>
+      <c r="T33" s="27" t="inlineStr">
+        <is>
+          <t>CLEAR_TARGETS</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="n">
@@ -3311,50 +3327,61 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Đạt điểm</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 4 ô đích</t>
+          <t>Đạt 600 điểm (nhiều đá hơn)</t>
         </is>
       </c>
       <c r="H34" s="5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I34" s="5" t="n">
         <v>2</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L34" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="M34" s="5" t="n">
-        <v>11</v>
+      <c r="M34" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N34" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O34" s="5" t="n">
-        <v>11</v>
+        <v>920</v>
       </c>
       <c r="P34" s="5" t="n">
-        <v>13</v>
+        <v>760</v>
       </c>
       <c r="Q34" s="5" t="n">
-        <v>15</v>
+        <v>600</v>
       </c>
       <c r="R34" s="5" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="S34" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="S34" s="4" t="inlineStr">
+        <is>
+          <t>Nhiều đá hơn</t>
+        </is>
+      </c>
+      <c r="T34" s="27" t="inlineStr">
+        <is>
+          <t>REACH_SCORE</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="12" t="n">
@@ -3382,50 +3409,61 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Hỗn hợp</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 4 ô đích</t>
+          <t>Phá 2 cổ vật + đạt 450 điểm</t>
         </is>
       </c>
       <c r="H35" s="5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I35" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J35" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K35" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="J35" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="K35" s="5" t="n">
-        <v>4</v>
-      </c>
       <c r="L35" s="5" t="n">
-        <v>21</v>
-      </c>
-      <c r="M35" s="5" t="n">
-        <v>11</v>
+        <v>20</v>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N35" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O35" s="5" t="n">
-        <v>11</v>
+        <v>720</v>
       </c>
       <c r="P35" s="5" t="n">
-        <v>13</v>
+        <v>580</v>
       </c>
       <c r="Q35" s="5" t="n">
-        <v>15</v>
+        <v>450</v>
       </c>
       <c r="R35" s="5" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="S35" s="4" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="S35" s="4" t="inlineStr">
+        <is>
+          <t>Cổ vật + điểm</t>
+        </is>
+      </c>
+      <c r="T35" s="27" t="inlineStr">
+        <is>
+          <t>MIXED</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="12" t="n">
@@ -3453,25 +3491,25 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Phá cổ vật</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 4 ô đích</t>
+          <t>Phá 3 cổ vật (đá vây chặt, bắt buộc xoay)</t>
         </is>
       </c>
       <c r="H36" s="5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L36" s="5" t="n">
         <v>21</v>
@@ -3494,9 +3532,18 @@
         <v>15</v>
       </c>
       <c r="R36" s="5" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="S36" s="4" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="S36" s="4" t="inlineStr">
+        <is>
+          <t>Đá vây chặt — bắt buộc xoay</t>
+        </is>
+      </c>
+      <c r="T36" s="27" t="inlineStr">
+        <is>
+          <t>CLEAR_TARGETS</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="12" t="n">
@@ -3524,50 +3571,61 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Đạt điểm</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 5 ô đích</t>
+          <t>Đạt 350 điểm (màn thở)</t>
         </is>
       </c>
       <c r="H37" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I37" s="5" t="n">
         <v>3</v>
       </c>
       <c r="J37" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L37" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="M37" s="5" t="n">
-        <v>11</v>
+        <v>15</v>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N37" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O37" s="5" t="n">
-        <v>11</v>
+        <v>560</v>
       </c>
       <c r="P37" s="5" t="n">
-        <v>13</v>
+        <v>450</v>
       </c>
       <c r="Q37" s="5" t="n">
-        <v>15</v>
+        <v>350</v>
       </c>
       <c r="R37" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="S37" s="4" t="inlineStr"/>
+        <v>2.5</v>
+      </c>
+      <c r="S37" s="4" t="inlineStr">
+        <is>
+          <t>Màn thở</t>
+        </is>
+      </c>
+      <c r="T37" s="27" t="inlineStr">
+        <is>
+          <t>REACH_SCORE</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="12" t="n">
@@ -3595,31 +3653,31 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Phá cổ vật</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 5 ô đích</t>
+          <t>Phá 3 cổ vật (mê đá nhiều chướng ngại)</t>
         </is>
       </c>
       <c r="H38" s="5" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L38" s="5" t="n">
         <v>22</v>
       </c>
       <c r="M38" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N38" s="5" t="inlineStr">
         <is>
@@ -3627,18 +3685,27 @@
         </is>
       </c>
       <c r="O38" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P38" s="5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q38" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R38" s="5" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="S38" s="4" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="S38" s="4" t="inlineStr">
+        <is>
+          <t>Mê đá — nhiều chướng ngại</t>
+        </is>
+      </c>
+      <c r="T38" s="27" t="inlineStr">
+        <is>
+          <t>CLEAR_TARGETS</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="12" t="n">
@@ -3666,50 +3733,61 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Đạt điểm</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 5 ô đích</t>
+          <t>Đạt 700 điểm (mật độ đá cao)</t>
         </is>
       </c>
       <c r="H39" s="5" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I39" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J39" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L39" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="M39" s="5" t="n">
-        <v>11</v>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N39" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O39" s="5" t="n">
-        <v>11</v>
+        <v>1080</v>
       </c>
       <c r="P39" s="5" t="n">
-        <v>13</v>
+        <v>900</v>
       </c>
       <c r="Q39" s="5" t="n">
-        <v>15</v>
+        <v>700</v>
       </c>
       <c r="R39" s="5" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="S39" s="4" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="S39" s="4" t="inlineStr">
+        <is>
+          <t>Mật độ đá cao</t>
+        </is>
+      </c>
+      <c r="T39" s="27" t="inlineStr">
+        <is>
+          <t>REACH_SCORE</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="12" t="n">
@@ -3737,50 +3815,61 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Hỗn hợp</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 6 ô đích</t>
+          <t>Phá 3 cổ vật + đạt 500 điểm</t>
         </is>
       </c>
       <c r="H40" s="5" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J40" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L40" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="M40" s="5" t="n">
-        <v>11</v>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N40" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Điểm</t>
         </is>
       </c>
       <c r="O40" s="5" t="n">
-        <v>11</v>
+        <v>800</v>
       </c>
       <c r="P40" s="5" t="n">
-        <v>13</v>
+        <v>650</v>
       </c>
       <c r="Q40" s="5" t="n">
-        <v>15</v>
+        <v>500</v>
       </c>
       <c r="R40" s="5" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="S40" s="4" t="inlineStr"/>
+        <v>4.5</v>
+      </c>
+      <c r="S40" s="4" t="inlineStr">
+        <is>
+          <t>Tổng hợp cổ vật + điểm</t>
+        </is>
+      </c>
+      <c r="T40" s="27" t="inlineStr">
+        <is>
+          <t>MIXED</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="12" t="n">
@@ -3808,50 +3897,61 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
+          <t>Boss combo</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Phá hết 7 ô đích</t>
+          <t>Tượng Cát Cổ (máu 12): giáp đá hồi +1 mỗi 2 lượt không bị đánh; combo ≥×2 gây (bậc−1) sát thương</t>
         </is>
       </c>
       <c r="H41" s="5" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J41" s="5" t="n">
         <v>8</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L41" s="5" t="n">
-        <v>27</v>
-      </c>
-      <c r="M41" s="5" t="n">
-        <v>11</v>
+        <v>22</v>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N41" s="5" t="inlineStr">
         <is>
-          <t>Nước</t>
+          <t>Combo</t>
         </is>
       </c>
       <c r="O41" s="5" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="P41" s="5" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="Q41" s="5" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="R41" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="S41" s="4" t="inlineStr"/>
+        <v>4.5</v>
+      </c>
+      <c r="S41" s="4" t="inlineStr">
+        <is>
+          <t>Boss Tượng Cát Cổ (Lõi Giáp — giáp đá hồi)</t>
+        </is>
+      </c>
+      <c r="T41" s="27" t="inlineStr">
+        <is>
+          <t>BOSS_COMBO</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="n">
@@ -8352,16 +8452,18 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Đá cố định làm chướng ngại</t>
+          <t>ĐÁ CỐ ĐỊNH chia bàn (nhẹ code — tái dùng STONE) + ô đích cổ vật; luyện xoay lách địa hình</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Clear ô đích</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>2</v>
+          <t>Điểm + Cổ vật + Boss</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>2–4</t>
+        </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>

</xml_diff>